<commit_message>
word doc and file orginzation
</commit_message>
<xml_diff>
--- a/Fall 2025/Controls Lab/Lab 2/outputs/tables/lab2_summary.xlsx
+++ b/Fall 2025/Controls Lab/Lab 2/outputs/tables/lab2_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,65 +436,75 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>run_index</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>controller</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>waveform</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>error_mean</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>error_std</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>error_rms</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>command_mean</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>command_std</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>command_rms</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>cycle_duration</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>rise_time_10_90</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>percent_overshoot</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>settling_time_2pct</t>
         </is>
@@ -508,279 +518,1091 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>BB_Sine_data</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>bang-bang</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>sine</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>0.1307781015579934</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>6.746862444837927</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>6.747264921977462</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>62.85114167333333</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>30.51976822651214</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>69.86761357957543</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>1.999271999999999</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>3900</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BB_Square_Data.xlsx</t>
+          <t>BB_Sine_data.xlsx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>BB_Sine_data</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>bang-bang</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>square</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0.2171694424598112</v>
-      </c>
-      <c r="E3" t="n">
-        <v>61.66705692919419</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>sine</t>
+        </is>
       </c>
       <c r="F3" t="n">
-        <v>61.66350537214049</v>
+        <v>0.03386959177161172</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.3536616483796887</v>
+        <v>3.829390244060211</v>
       </c>
       <c r="H3" t="n">
-        <v>99.00568424882476</v>
+        <v>3.8290495666924</v>
       </c>
       <c r="I3" t="n">
-        <v>99</v>
+        <v>62.88297898642418</v>
       </c>
       <c r="J3" t="n">
-        <v>3.999580999999999</v>
+        <v>30.41088763304329</v>
       </c>
       <c r="K3" t="n">
-        <v>7838</v>
+        <v>69.84879556537329</v>
       </c>
       <c r="L3" t="n">
-        <v>0.3178000000000001</v>
+        <v>1.999127999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>105.1764126262626</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.4531809999999989</v>
-      </c>
+        <v>3904</v>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PID_Sine_KP_Data.xlsx</t>
+          <t>BB_Sine_data.xlsx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>pid</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+          <t>BB_Sine_data</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>sine</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>46.55690632584561</v>
-      </c>
-      <c r="E4" t="n">
-        <v>30.4276074395317</v>
-      </c>
       <c r="F4" t="n">
-        <v>55.61604674275816</v>
+        <v>1.648218131966715</v>
       </c>
       <c r="G4" t="n">
-        <v>62.95032997483787</v>
+        <v>7.698315915572156</v>
       </c>
       <c r="H4" t="n">
-        <v>30.42764680652277</v>
+        <v>7.87180599365697</v>
       </c>
       <c r="I4" t="n">
-        <v>69.91670449661419</v>
+        <v>62.89271330196993</v>
       </c>
       <c r="J4" t="n">
-        <v>1.999791</v>
+        <v>30.5099231658106</v>
       </c>
       <c r="K4" t="n">
-        <v>3855</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+        <v>69.90069755589413</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1.999456999999992</v>
+      </c>
+      <c r="M4" t="n">
+        <v>3858</v>
+      </c>
       <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PID_Square_KP_Data.xlsx</t>
+          <t>BB_Sine_data.xlsx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>pid</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>square</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>-15.79590864787465</v>
-      </c>
-      <c r="E5" t="n">
-        <v>99.00455395931397</v>
+          <t>BB_Sine_data</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>sine</t>
+        </is>
       </c>
       <c r="F5" t="n">
-        <v>100.2504547755771</v>
+        <v>-0.2158783434629362</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5975343521253371</v>
+        <v>14.70690837205359</v>
       </c>
       <c r="H5" t="n">
-        <v>99.00455395931397</v>
+        <v>14.70660968923022</v>
       </c>
       <c r="I5" t="n">
-        <v>99</v>
+        <v>63.11097382740076</v>
       </c>
       <c r="J5" t="n">
-        <v>3.999683000000001</v>
+        <v>30.45562215927638</v>
       </c>
       <c r="K5" t="n">
-        <v>7787</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
+        <v>70.07355001027753</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1.999746999999999</v>
+      </c>
       <c r="M5" t="n">
-        <v>58.27951666666647</v>
+        <v>3905</v>
       </c>
       <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PID_ack_tuning.xlsx</t>
+          <t>BB_Sine_data.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>pid</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>square</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0.5295785898352671</v>
-      </c>
-      <c r="E6" t="n">
-        <v>47.48944598132193</v>
+          <t>BB_Sine_data</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>sine</t>
+        </is>
       </c>
       <c r="F6" t="n">
-        <v>47.48936663483696</v>
+        <v>-0.5172086918104386</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.4424722257693781</v>
+        <v>13.04109235492207</v>
       </c>
       <c r="H6" t="n">
-        <v>99.00533277285273</v>
+        <v>13.04966995978054</v>
       </c>
       <c r="I6" t="n">
-        <v>99</v>
+        <v>63.17347611770753</v>
       </c>
       <c r="J6" t="n">
-        <v>3.999129</v>
+        <v>30.43791852203713</v>
       </c>
       <c r="K6" t="n">
-        <v>7831</v>
+        <v>70.1221567242779</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1593400000000003</v>
+        <v>1.999513000000007</v>
       </c>
       <c r="M6" t="n">
-        <v>103.3299015151515</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.2528869999999994</v>
-      </c>
+        <v>3891</v>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>BB_Sine_data.xlsx</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BB_Sine_data</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>sine</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.8381406836055278</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6.137834251069425</v>
+      </c>
+      <c r="H7" t="n">
+        <v>6.194005276041231</v>
+      </c>
+      <c r="I7" t="n">
+        <v>62.76678957417511</v>
+      </c>
+      <c r="J7" t="n">
+        <v>30.45421033669139</v>
+      </c>
+      <c r="K7" t="n">
+        <v>69.76308364507896</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1.999597000000023</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3849</v>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BB_Square_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BB_Square_Data</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0.2171694424598112</v>
+      </c>
+      <c r="G8" t="n">
+        <v>61.66705692919419</v>
+      </c>
+      <c r="H8" t="n">
+        <v>61.66350537214049</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-0.3536616483796887</v>
+      </c>
+      <c r="J8" t="n">
+        <v>99.00568424882476</v>
+      </c>
+      <c r="K8" t="n">
+        <v>99</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3.999580999999999</v>
+      </c>
+      <c r="M8" t="n">
+        <v>7838</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.3178000000000001</v>
+      </c>
+      <c r="O8" t="n">
+        <v>105.1764126262626</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.4531809999999989</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BB_Square_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BB_Square_Data</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>-2.082320329666109</v>
+      </c>
+      <c r="G9" t="n">
+        <v>59.49297069287311</v>
+      </c>
+      <c r="H9" t="n">
+        <v>59.52559815479506</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-0.2152999872073686</v>
+      </c>
+      <c r="J9" t="n">
+        <v>99.00609883339499</v>
+      </c>
+      <c r="K9" t="n">
+        <v>99</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3.999136999999997</v>
+      </c>
+      <c r="M9" t="n">
+        <v>7817</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.3121799999999979</v>
+      </c>
+      <c r="O9" t="n">
+        <v>104.9055176767677</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.4313079999999943</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BB_Square_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BB_Square_Data</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.04430504494382174</v>
+      </c>
+      <c r="G10" t="n">
+        <v>60.53139607048872</v>
+      </c>
+      <c r="H10" t="n">
+        <v>60.52754779847156</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-0.07584269662921349</v>
+      </c>
+      <c r="J10" t="n">
+        <v>99.00629177707135</v>
+      </c>
+      <c r="K10" t="n">
+        <v>99</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3.999852999999987</v>
+      </c>
+      <c r="M10" t="n">
+        <v>7832</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.3081449999999961</v>
+      </c>
+      <c r="O10" t="n">
+        <v>103.0827343434344</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.4311069999999972</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BB_Square_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BB_Square_Data</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0.8367232466051767</v>
+      </c>
+      <c r="G11" t="n">
+        <v>44.32782532691257</v>
+      </c>
+      <c r="H11" t="n">
+        <v>44.33288260636675</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.1775557263643351</v>
+      </c>
+      <c r="J11" t="n">
+        <v>99.00618265254444</v>
+      </c>
+      <c r="K11" t="n">
+        <v>99</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3.999791999999999</v>
+      </c>
+      <c r="M11" t="n">
+        <v>7806</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.2117129999999889</v>
+      </c>
+      <c r="O11" t="n">
+        <v>113.781744949495</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.2257919999999984</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BB_Square_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BB_Square_Data</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>-0.1766442675786243</v>
+      </c>
+      <c r="G12" t="n">
+        <v>41.12886652036722</v>
+      </c>
+      <c r="H12" t="n">
+        <v>41.12661674281817</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-0.2278189721298901</v>
+      </c>
+      <c r="J12" t="n">
+        <v>99.00606676581354</v>
+      </c>
+      <c r="K12" t="n">
+        <v>99</v>
+      </c>
+      <c r="L12" t="n">
+        <v>3.999517999999995</v>
+      </c>
+      <c r="M12" t="n">
+        <v>7822</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.1677620000000104</v>
+      </c>
+      <c r="O12" t="n">
+        <v>114.2253171717173</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.2033830000000023</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BB_Square_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BB_Square_Data</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>bang-bang</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>-5.751548972876153</v>
+      </c>
+      <c r="G13" t="n">
+        <v>46.82489609807027</v>
+      </c>
+      <c r="H13" t="n">
+        <v>47.17383476867705</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.05066530194472876</v>
+      </c>
+      <c r="J13" t="n">
+        <v>99.00632080517977</v>
+      </c>
+      <c r="K13" t="n">
+        <v>99</v>
+      </c>
+      <c r="L13" t="n">
+        <v>3.999392</v>
+      </c>
+      <c r="M13" t="n">
+        <v>7816</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.1508480000000247</v>
+      </c>
+      <c r="O13" t="n">
+        <v>114.631794949495</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.2257619999999747</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PID_Sine_KP_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PID_Sine_KP_Data</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>pid</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>sine</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>46.55690632584561</v>
+      </c>
+      <c r="G14" t="n">
+        <v>30.4276074395317</v>
+      </c>
+      <c r="H14" t="n">
+        <v>55.61604674275816</v>
+      </c>
+      <c r="I14" t="n">
+        <v>62.95032997483787</v>
+      </c>
+      <c r="J14" t="n">
+        <v>30.42764680652277</v>
+      </c>
+      <c r="K14" t="n">
+        <v>69.91670449661419</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1.999791</v>
+      </c>
+      <c r="M14" t="n">
+        <v>3855</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PID_Sine_KP_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PID_Sine_KP_Data</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>pid</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>sine</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>46.78938715579188</v>
+      </c>
+      <c r="G15" t="n">
+        <v>37.43956209468907</v>
+      </c>
+      <c r="H15" t="n">
+        <v>59.92168956578168</v>
+      </c>
+      <c r="I15" t="n">
+        <v>63.14373774155579</v>
+      </c>
+      <c r="J15" t="n">
+        <v>30.40190996398426</v>
+      </c>
+      <c r="K15" t="n">
+        <v>70.07974911983742</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1.999488999999997</v>
+      </c>
+      <c r="M15" t="n">
+        <v>3908</v>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PID_Sine_KP_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PID_Sine_KP_Data</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>pid</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>sine</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>12.34140930423265</v>
+      </c>
+      <c r="G16" t="n">
+        <v>28.49687624438192</v>
+      </c>
+      <c r="H16" t="n">
+        <v>31.05114545546492</v>
+      </c>
+      <c r="I16" t="n">
+        <v>62.87947363068619</v>
+      </c>
+      <c r="J16" t="n">
+        <v>30.52099255152449</v>
+      </c>
+      <c r="K16" t="n">
+        <v>69.89363192613904</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1.999459999999999</v>
+      </c>
+      <c r="M16" t="n">
+        <v>3891</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PID_Square_KP_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PID_Square_KP_Data</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>pid</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>-15.79590864787465</v>
+      </c>
+      <c r="G17" t="n">
+        <v>99.00455395931397</v>
+      </c>
+      <c r="H17" t="n">
+        <v>100.2504547755771</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.5975343521253371</v>
+      </c>
+      <c r="J17" t="n">
+        <v>99.00455395931397</v>
+      </c>
+      <c r="K17" t="n">
+        <v>99</v>
+      </c>
+      <c r="L17" t="n">
+        <v>3.999683000000001</v>
+      </c>
+      <c r="M17" t="n">
+        <v>7787</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="n">
+        <v>58.27951666666647</v>
+      </c>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PID_Square_KP_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PID_Square_KP_Data</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>pid</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.9029190072983379</v>
+      </c>
+      <c r="G18" t="n">
+        <v>70.2948463570617</v>
+      </c>
+      <c r="H18" t="n">
+        <v>70.29614491463396</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.07605633802816901</v>
+      </c>
+      <c r="J18" t="n">
+        <v>99.00630942002199</v>
+      </c>
+      <c r="K18" t="n">
+        <v>99</v>
+      </c>
+      <c r="L18" t="n">
+        <v>3.999482</v>
+      </c>
+      <c r="M18" t="n">
+        <v>7810</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="n">
+        <v>79.5619393939393</v>
+      </c>
+      <c r="P18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PID_Square_KP_Data.xlsx</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PID_Square_KP_Data</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>pid</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0.3613156400154512</v>
+      </c>
+      <c r="G19" t="n">
+        <v>46.91544086932835</v>
+      </c>
+      <c r="H19" t="n">
+        <v>46.91381198555156</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-0.2676709154113557</v>
+      </c>
+      <c r="J19" t="n">
+        <v>99.00601185137839</v>
+      </c>
+      <c r="K19" t="n">
+        <v>99</v>
+      </c>
+      <c r="L19" t="n">
+        <v>3.999536999999989</v>
+      </c>
+      <c r="M19" t="n">
+        <v>7767</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.4702529999999996</v>
+      </c>
+      <c r="O19" t="n">
+        <v>92.14698585858582</v>
+      </c>
+      <c r="P19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PID_ack_tuning.xlsx</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PID_ack_tuning</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>pid</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>square</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.5295785898352671</v>
+      </c>
+      <c r="G20" t="n">
+        <v>47.48944598132193</v>
+      </c>
+      <c r="H20" t="n">
+        <v>47.48936663483696</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-0.4424722257693781</v>
+      </c>
+      <c r="J20" t="n">
+        <v>99.00533277285273</v>
+      </c>
+      <c r="K20" t="n">
+        <v>99</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3.999129</v>
+      </c>
+      <c r="M20" t="n">
+        <v>7831</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.1593400000000003</v>
+      </c>
+      <c r="O20" t="n">
+        <v>103.3299015151515</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.2528869999999994</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>PID_manual_tuning.xlsx</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PID_manual_tuning_better</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>pid</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>square</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="F21" t="n">
         <v>-0.05431368437900547</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G21" t="n">
         <v>43.87596777460819</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H21" t="n">
         <v>43.87319234324355</v>
       </c>
-      <c r="G7" t="n">
+      <c r="I21" t="n">
         <v>-0.4056338028169014</v>
       </c>
-      <c r="H7" t="n">
+      <c r="J21" t="n">
         <v>99.00550757623566</v>
       </c>
-      <c r="I7" t="n">
+      <c r="K21" t="n">
         <v>99</v>
       </c>
-      <c r="J7" t="n">
+      <c r="L21" t="n">
         <v>3.999536999999975</v>
       </c>
-      <c r="K7" t="n">
+      <c r="M21" t="n">
         <v>7810</v>
       </c>
-      <c r="L7" t="n">
+      <c r="N21" t="n">
         <v>0.1534700000000271</v>
       </c>
-      <c r="M7" t="n">
+      <c r="O21" t="n">
         <v>109.5258151515152</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P21" t="n">
         <v>0.2237129999999752</v>
       </c>
     </row>

</xml_diff>